<commit_message>
Update MASTER.xlsx in data folder
</commit_message>
<xml_diff>
--- a/data/MASTER.xlsx
+++ b/data/MASTER.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1159">
   <si>
     <t>This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -3440,6 +3440,27 @@
   </si>
   <si>
     <t>YASH LASERTEK INDIA</t>
+  </si>
+  <si>
+    <t>V K TRAVELS &amp; SERVICES</t>
+  </si>
+  <si>
+    <t>2 X 2 LOGISTICS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>NEW GRIP</t>
+  </si>
+  <si>
+    <t>SANGITAM TRAVELS PVT LTD</t>
+  </si>
+  <si>
+    <t>PRATIKSHA FREIGHTS CARRIERS</t>
+  </si>
+  <si>
+    <t>WAMAN’S RUBBER LLP</t>
+  </si>
+  <si>
+    <t>AILSANGHANI</t>
   </si>
   <si>
     <t xml:space="preserve">Vehicle Type </t>
@@ -3791,7 +3812,7 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
@@ -3945,7 +3966,10 @@
     <xf numFmtId="49" fontId="8" fillId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="4" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -3957,16 +3981,16 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -5212,7 +5236,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I793"/>
+  <dimension ref="A1:I795"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="19" style="25" customWidth="1"/>
@@ -27929,61 +27953,83 @@
       </c>
     </row>
     <row r="791" ht="13.55" customHeight="1">
-      <c r="A791" t="s" s="35">
+      <c r="A791" t="s" s="31">
         <v>1067</v>
       </c>
-      <c r="B791" t="s" s="35">
+      <c r="B791" t="s" s="31">
         <v>1068</v>
       </c>
-      <c r="C791" s="36">
+      <c r="C791" s="32">
         <v>29</v>
       </c>
-      <c r="D791" t="s" s="35">
-        <v>23</v>
-      </c>
-      <c r="E791" t="s" s="35">
+      <c r="D791" t="s" s="31">
+        <v>23</v>
+      </c>
+      <c r="E791" t="s" s="31">
         <v>1069</v>
       </c>
-      <c r="F791" t="s" s="35">
-        <v>25</v>
-      </c>
-      <c r="G791" s="36">
-        <v>0</v>
-      </c>
-      <c r="H791" t="s" s="35">
-        <v>26</v>
-      </c>
-      <c r="I791" s="36">
+      <c r="F791" t="s" s="31">
+        <v>25</v>
+      </c>
+      <c r="G791" s="32">
+        <v>0</v>
+      </c>
+      <c r="H791" t="s" s="31">
+        <v>26</v>
+      </c>
+      <c r="I791" s="32">
         <v>0</v>
       </c>
     </row>
     <row r="792" ht="13.55" customHeight="1">
-      <c r="A792" s="37"/>
-      <c r="B792" s="38"/>
-      <c r="C792" s="39">
+      <c r="A792" s="31"/>
+      <c r="B792" s="31"/>
+      <c r="C792" s="32"/>
+      <c r="D792" s="31"/>
+      <c r="E792" s="31"/>
+      <c r="F792" s="31"/>
+      <c r="G792" s="32"/>
+      <c r="H792" s="31"/>
+      <c r="I792" s="32"/>
+    </row>
+    <row r="793" ht="13.55" customHeight="1">
+      <c r="A793" s="35"/>
+      <c r="B793" s="35"/>
+      <c r="C793" s="36"/>
+      <c r="D793" s="35"/>
+      <c r="E793" s="35"/>
+      <c r="F793" s="35"/>
+      <c r="G793" s="36"/>
+      <c r="H793" s="35"/>
+      <c r="I793" s="36"/>
+    </row>
+    <row r="794" ht="13.55" customHeight="1">
+      <c r="A794" s="37"/>
+      <c r="B794" s="38"/>
+      <c r="C794" s="39">
         <v>9330.530000000001</v>
       </c>
-      <c r="D792" s="38"/>
-      <c r="E792" s="38"/>
-      <c r="F792" s="38"/>
-      <c r="G792" s="38"/>
-      <c r="H792" s="38"/>
-      <c r="I792" s="40">
+      <c r="D794" s="38"/>
+      <c r="E794" s="38"/>
+      <c r="F794" s="38"/>
+      <c r="G794" s="38"/>
+      <c r="H794" s="38"/>
+      <c r="I794" s="40">
         <v>1101.1</v>
       </c>
     </row>
-    <row r="793" ht="13.55" customHeight="1">
-      <c r="A793" s="41"/>
-      <c r="B793" s="42"/>
-      <c r="C793" s="43">
+    <row r="795" ht="13.55" customHeight="1">
+      <c r="A795" s="41"/>
+      <c r="B795" s="42"/>
+      <c r="C795" s="43">
         <v>11186</v>
       </c>
-      <c r="D793" s="42"/>
-      <c r="E793" s="42"/>
-      <c r="F793" s="42"/>
-      <c r="G793" s="42"/>
-      <c r="H793" s="42"/>
-      <c r="I793" s="44">
+      <c r="D795" s="42"/>
+      <c r="E795" s="42"/>
+      <c r="F795" s="42"/>
+      <c r="G795" s="42"/>
+      <c r="H795" s="42"/>
+      <c r="I795" s="44">
         <v>1394</v>
       </c>
     </row>
@@ -27998,7 +28044,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12" style="45" customWidth="1"/>
@@ -28775,21 +28821,121 @@
       </c>
     </row>
     <row r="46" ht="13.65" customHeight="1">
-      <c r="A46" s="51">
+      <c r="A46" s="48">
         <v>1404896</v>
       </c>
-      <c r="B46" t="s" s="52">
+      <c r="B46" t="s" s="49">
         <v>1133</v>
       </c>
-      <c r="C46" t="s" s="53">
+      <c r="C46" t="s" s="50">
         <v>1076</v>
       </c>
-      <c r="D46" s="51">
+      <c r="D46" s="48">
         <v>7290024942</v>
       </c>
-      <c r="E46" t="s" s="52">
+      <c r="E46" t="s" s="49">
         <v>1079</v>
       </c>
+    </row>
+    <row r="47" ht="13.65" customHeight="1">
+      <c r="A47" s="48">
+        <v>1122689</v>
+      </c>
+      <c r="B47" t="s" s="49">
+        <v>1134</v>
+      </c>
+      <c r="C47" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D47" s="51"/>
+      <c r="E47" t="s" s="49">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="48" ht="13.65" customHeight="1">
+      <c r="A48" s="48">
+        <v>1908197</v>
+      </c>
+      <c r="B48" t="s" s="49">
+        <v>1135</v>
+      </c>
+      <c r="C48" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D48" s="51"/>
+      <c r="E48" s="49"/>
+    </row>
+    <row r="49" ht="13.65" customHeight="1">
+      <c r="A49" s="48">
+        <v>2501387</v>
+      </c>
+      <c r="B49" t="s" s="49">
+        <v>1136</v>
+      </c>
+      <c r="C49" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D49" s="51"/>
+      <c r="E49" s="49"/>
+    </row>
+    <row r="50" ht="13.65" customHeight="1">
+      <c r="A50" s="51"/>
+      <c r="B50" t="s" s="49">
+        <v>1137</v>
+      </c>
+      <c r="C50" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D50" s="51"/>
+      <c r="E50" s="49"/>
+    </row>
+    <row r="51" ht="13.65" customHeight="1">
+      <c r="A51" s="48">
+        <v>1907821</v>
+      </c>
+      <c r="B51" t="s" s="49">
+        <v>1138</v>
+      </c>
+      <c r="C51" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D51" s="51"/>
+      <c r="E51" s="49"/>
+    </row>
+    <row r="52" ht="13.65" customHeight="1">
+      <c r="A52" s="48">
+        <v>2501969</v>
+      </c>
+      <c r="B52" t="s" s="49">
+        <v>1139</v>
+      </c>
+      <c r="C52" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D52" s="51"/>
+      <c r="E52" t="s" s="49">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="53" ht="13.65" customHeight="1">
+      <c r="A53" s="51"/>
+      <c r="B53" t="s" s="49">
+        <v>1140</v>
+      </c>
+      <c r="C53" t="s" s="50">
+        <v>1076</v>
+      </c>
+      <c r="D53" s="51"/>
+      <c r="E53" s="49"/>
+    </row>
+    <row r="54" ht="13.65" customHeight="1">
+      <c r="A54" s="52"/>
+      <c r="B54" s="53"/>
+      <c r="C54" t="s" s="54">
+        <v>1076</v>
+      </c>
+      <c r="D54" s="52"/>
+      <c r="E54" s="53"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -28808,238 +28954,238 @@
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="5" width="16.3516" style="54" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="54" customWidth="1"/>
+    <col min="1" max="5" width="16.3516" style="55" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="55" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.1" customHeight="1">
-      <c r="A1" t="s" s="55">
+      <c r="A1" t="s" s="56">
         <v>10</v>
       </c>
-      <c r="B1" t="s" s="55">
-        <v>1134</v>
-      </c>
-      <c r="C1" t="s" s="55">
-        <v>1135</v>
-      </c>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
+      <c r="B1" t="s" s="56">
+        <v>1141</v>
+      </c>
+      <c r="C1" t="s" s="56">
+        <v>1142</v>
+      </c>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
     </row>
     <row r="2" ht="12.9" customHeight="1">
-      <c r="A2" t="s" s="57">
+      <c r="A2" t="s" s="58">
         <v>1077</v>
       </c>
-      <c r="B2" t="s" s="57">
-        <v>1136</v>
-      </c>
-      <c r="C2" t="s" s="57">
-        <v>1137</v>
-      </c>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
+      <c r="B2" t="s" s="58">
+        <v>1143</v>
+      </c>
+      <c r="C2" t="s" s="58">
+        <v>1144</v>
+      </c>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
     </row>
     <row r="3" ht="12.9" customHeight="1">
-      <c r="A3" t="s" s="57">
+      <c r="A3" t="s" s="58">
         <v>1079</v>
       </c>
-      <c r="B3" t="s" s="57">
-        <v>1138</v>
-      </c>
-      <c r="C3" t="s" s="57">
-        <v>1139</v>
-      </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
+      <c r="B3" t="s" s="58">
+        <v>1145</v>
+      </c>
+      <c r="C3" t="s" s="58">
+        <v>1146</v>
+      </c>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
     </row>
     <row r="4" ht="12.9" customHeight="1">
-      <c r="A4" t="s" s="57">
+      <c r="A4" t="s" s="58">
         <v>1081</v>
       </c>
-      <c r="B4" t="s" s="57">
-        <v>1140</v>
-      </c>
-      <c r="C4" t="s" s="57">
-        <v>1141</v>
-      </c>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
+      <c r="B4" t="s" s="58">
+        <v>1147</v>
+      </c>
+      <c r="C4" t="s" s="58">
+        <v>1148</v>
+      </c>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
     </row>
     <row r="5" ht="12.9" customHeight="1">
-      <c r="A5" t="s" s="57">
+      <c r="A5" t="s" s="58">
         <v>1083</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" t="s" s="57">
-        <v>1142</v>
-      </c>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" t="s" s="58">
+        <v>1149</v>
+      </c>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
     </row>
     <row r="6" ht="12.9" customHeight="1">
-      <c r="A6" t="s" s="57">
+      <c r="A6" t="s" s="58">
         <v>1085</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" t="s" s="57">
-        <v>1143</v>
-      </c>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
+      <c r="B6" s="59"/>
+      <c r="C6" t="s" s="58">
+        <v>1150</v>
+      </c>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
     </row>
     <row r="7" ht="12.9" customHeight="1">
-      <c r="A7" t="s" s="57">
+      <c r="A7" t="s" s="58">
         <v>1088</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" t="s" s="57">
-        <v>1139</v>
-      </c>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58"/>
+      <c r="B7" s="59"/>
+      <c r="C7" t="s" s="58">
+        <v>1146</v>
+      </c>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
     </row>
     <row r="8" ht="12.9" customHeight="1">
-      <c r="A8" t="s" s="57">
+      <c r="A8" t="s" s="58">
         <v>1089</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" t="s" s="57">
-        <v>1144</v>
-      </c>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
+      <c r="B8" s="59"/>
+      <c r="C8" t="s" s="58">
+        <v>1151</v>
+      </c>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
     </row>
     <row r="9" ht="12.9" customHeight="1">
-      <c r="A9" t="s" s="57">
-        <v>1145</v>
-      </c>
-      <c r="B9" s="58"/>
-      <c r="C9" t="s" s="57">
-        <v>1146</v>
-      </c>
-      <c r="D9" s="58"/>
-      <c r="E9" s="58"/>
+      <c r="A9" t="s" s="58">
+        <v>1152</v>
+      </c>
+      <c r="B9" s="59"/>
+      <c r="C9" t="s" s="58">
+        <v>1153</v>
+      </c>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
     </row>
     <row r="10" ht="12.9" customHeight="1">
-      <c r="A10" t="s" s="57">
+      <c r="A10" t="s" s="58">
         <v>1093</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" t="s" s="57">
-        <v>1147</v>
-      </c>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
+      <c r="B10" s="59"/>
+      <c r="C10" t="s" s="58">
+        <v>1154</v>
+      </c>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
     </row>
     <row r="11" ht="12.9" customHeight="1">
-      <c r="A11" t="s" s="57">
+      <c r="A11" t="s" s="58">
         <v>1096</v>
       </c>
-      <c r="B11" s="58"/>
-      <c r="C11" t="s" s="57">
-        <v>1148</v>
-      </c>
-      <c r="D11" s="58"/>
-      <c r="E11" s="58"/>
+      <c r="B11" s="59"/>
+      <c r="C11" t="s" s="58">
+        <v>1155</v>
+      </c>
+      <c r="D11" s="59"/>
+      <c r="E11" s="59"/>
     </row>
     <row r="12" ht="12.9" customHeight="1">
-      <c r="A12" t="s" s="57">
+      <c r="A12" t="s" s="58">
         <v>1101</v>
       </c>
-      <c r="B12" s="58"/>
-      <c r="C12" t="s" s="57">
-        <v>1149</v>
-      </c>
-      <c r="D12" s="58"/>
-      <c r="E12" s="58"/>
+      <c r="B12" s="59"/>
+      <c r="C12" t="s" s="58">
+        <v>1156</v>
+      </c>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
     </row>
     <row r="13" ht="12.9" customHeight="1">
-      <c r="A13" t="s" s="57">
+      <c r="A13" t="s" s="58">
         <v>1103</v>
       </c>
-      <c r="B13" s="58"/>
-      <c r="C13" t="s" s="57">
-        <v>1150</v>
-      </c>
-      <c r="D13" s="58"/>
-      <c r="E13" s="58"/>
+      <c r="B13" s="59"/>
+      <c r="C13" t="s" s="58">
+        <v>1157</v>
+      </c>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
     </row>
     <row r="14" ht="12.9" customHeight="1">
-      <c r="A14" t="s" s="57">
+      <c r="A14" t="s" s="58">
         <v>1109</v>
       </c>
-      <c r="B14" s="58"/>
-      <c r="C14" t="s" s="57">
-        <v>1151</v>
-      </c>
-      <c r="D14" s="58"/>
-      <c r="E14" s="58"/>
+      <c r="B14" s="59"/>
+      <c r="C14" t="s" s="58">
+        <v>1158</v>
+      </c>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
     </row>
     <row r="15" ht="12.9" customHeight="1">
-      <c r="A15" t="s" s="57">
+      <c r="A15" t="s" s="58">
         <v>1115</v>
       </c>
-      <c r="B15" s="58"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
+      <c r="B15" s="59"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
     </row>
     <row r="16" ht="12.9" customHeight="1">
-      <c r="A16" t="s" s="57">
+      <c r="A16" t="s" s="58">
         <v>1123</v>
       </c>
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="58"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
     </row>
     <row r="17" ht="12.9" customHeight="1">
-      <c r="A17" s="57"/>
-      <c r="B17" s="58"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="58"/>
-      <c r="E17" s="58"/>
+      <c r="A17" s="58"/>
+      <c r="B17" s="59"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
     </row>
     <row r="18" ht="12.9" customHeight="1">
-      <c r="A18" s="57"/>
-      <c r="B18" s="58"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="58"/>
-      <c r="E18" s="58"/>
+      <c r="A18" s="58"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
     </row>
     <row r="19" ht="12.9" customHeight="1">
-      <c r="A19" s="57"/>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
+      <c r="A19" s="58"/>
+      <c r="B19" s="59"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="59"/>
     </row>
     <row r="20" ht="12.9" customHeight="1">
-      <c r="A20" s="57"/>
-      <c r="B20" s="58"/>
-      <c r="C20" s="58"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="58"/>
+      <c r="A20" s="58"/>
+      <c r="B20" s="59"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
     </row>
     <row r="21" ht="12.9" customHeight="1">
-      <c r="A21" s="57"/>
-      <c r="B21" s="58"/>
-      <c r="C21" s="58"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="58"/>
+      <c r="A21" s="58"/>
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
     </row>
     <row r="22" ht="12.9" customHeight="1">
-      <c r="A22" s="57"/>
-      <c r="B22" s="58"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="58"/>
+      <c r="A22" s="58"/>
+      <c r="B22" s="59"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59"/>
     </row>
     <row r="23" ht="12.9" customHeight="1">
-      <c r="A23" s="57"/>
-      <c r="B23" s="58"/>
-      <c r="C23" s="58"/>
-      <c r="D23" s="58"/>
-      <c r="E23" s="58"/>
+      <c r="A23" s="58"/>
+      <c r="B23" s="59"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="59"/>
+      <c r="E23" s="59"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>